<commit_message>
docs: ajustar al corte del 12/09 las tareas del cronograma con fecha futura
42 tareas de los modulos 8 a 11 empezaban despues del corte y estaban al 100 %.
Revisadas contra el codigo: 34 siguen al 100 % como adelantadas (el codigo
esta en el repositorio desde el 17/08); 6 quedan al 50 % (protecciones
electricas fisicas e indicadores de humedad, temperatura, tendencia semanal y
comparacion entre periodos) y 2 al 0 % (conexion y modelo de Power BI, sin
.pbix). Avance ponderado 83.9 %; el modulo 11 pasa a Parcial.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Planificacion Victor Madrid Final.xlsx
+++ b/Planificacion Victor Madrid Final.xlsx
@@ -3696,7 +3696,7 @@
       </c>
       <c r="L80" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="L82" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -3810,7 +3810,7 @@
       </c>
       <c r="L83" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -3848,7 +3848,7 @@
       </c>
       <c r="L84" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -3890,7 +3890,7 @@
       </c>
       <c r="L85" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -3921,14 +3921,14 @@
         <v>46283</v>
       </c>
       <c r="J86" s="30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K86" s="4" t="n">
         <v>11</v>
       </c>
       <c r="L86" s="28" t="inlineStr">
         <is>
-          <t>Validado funcionalmente con simulador y contrato MQTT; instalación física incluida en el Módulo 12.</t>
+          <t>Parcial: parada de emergencia, sobrecorriente y bloqueo por marcha en seco implementados y probados en software. Las protecciones eléctricas físicas se instalan en el módulo 12.</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="L87" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -3997,14 +3997,14 @@
         <v>46286</v>
       </c>
       <c r="J88" s="30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K88" s="4" t="n">
         <v>12</v>
       </c>
       <c r="L88" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Parcial: pruebas automatizadas de las protecciones por software superadas; la prueba de las protecciones eléctricas físicas queda para el montaje del módulo 12.</t>
         </is>
       </c>
     </row>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="L89" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="L90" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="L91" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="L92" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4208,7 +4208,7 @@
       </c>
       <c r="L93" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="L94" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="L95" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="L96" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="L97" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="L98" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="L99" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="L100" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4530,7 +4530,7 @@
       </c>
       <c r="L101" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4568,7 +4568,7 @@
       </c>
       <c r="L102" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="L103" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4640,7 +4640,7 @@
       </c>
       <c r="L104" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="L105" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
       </c>
       <c r="L106" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="L107" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="L108" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4838,7 +4838,7 @@
       </c>
       <c r="L109" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4876,7 +4876,7 @@
       </c>
       <c r="L110" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4914,7 @@
       </c>
       <c r="L111" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4962,7 +4962,7 @@
       </c>
       <c r="L112" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -4993,14 +4993,14 @@
         <v>46304</v>
       </c>
       <c r="J113" s="30" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="K113" s="4" t="n">
         <v>14</v>
       </c>
       <c r="L113" s="28" t="inlineStr">
         <is>
-          <t>Modelo analítico, vistas, indicadores y guía reproducible completos; publicación productiva incluida en el Módulo 12.</t>
+          <t>Pendiente: Power BI Desktop no está instalado y no existe archivo .pbix. Las vistas SQL y el procedimiento de origen ya están listos (fila 112).</t>
         </is>
       </c>
     </row>
@@ -5027,14 +5027,14 @@
         <v>46307</v>
       </c>
       <c r="J114" s="30" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="K114" s="4" t="n">
         <v>14</v>
       </c>
       <c r="L114" s="28" t="inlineStr">
         <is>
-          <t>Modelo analítico, vistas, indicadores y guía reproducible completos; publicación productiva incluida en el Módulo 12.</t>
+          <t>Pendiente: el modelo, sus relaciones y las medidas DAX están especificados en docs/sprint6-reporting-audit-powerbi.md y en GET /api/week14/powerbi/model, pero no se han construido en Power BI.</t>
         </is>
       </c>
     </row>
@@ -5065,14 +5065,14 @@
         <v>46307</v>
       </c>
       <c r="J115" s="30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K115" s="4" t="n">
         <v>15</v>
       </c>
       <c r="L115" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Parcial: las vistas analíticas tienen prueba automatizada; la conexión y el modelo de Power BI no pueden probarse hasta construirse (filas 113 y 114).</t>
         </is>
       </c>
     </row>
@@ -5107,14 +5107,14 @@
         <v>46309</v>
       </c>
       <c r="J116" s="30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K116" s="4" t="n">
         <v>15</v>
       </c>
       <c r="L116" s="28" t="inlineStr">
         <is>
-          <t>Modelo analítico, vistas, indicadores y guía reproducible completos; publicación productiva incluida en el Módulo 12.</t>
+          <t>Parcial: el dashboard web muestra consumo, costo y eficiencia por cultivo. Faltan los indicadores analíticos de humedad y temperatura.</t>
         </is>
       </c>
     </row>
@@ -5141,14 +5141,14 @@
         <v>46309</v>
       </c>
       <c r="J117" s="30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K117" s="4" t="n">
         <v>15</v>
       </c>
       <c r="L117" s="28" t="inlineStr">
         <is>
-          <t>Modelo analítico, vistas, indicadores y guía reproducible completos; publicación productiva incluida en el Módulo 12.</t>
+          <t>Parcial: la tendencia diaria está en pantalla y la API calcula la semanal, pero la pantalla no la muestra y no existe comparación entre periodos.</t>
         </is>
       </c>
     </row>
@@ -5182,7 +5182,7 @@
       </c>
       <c r="L118" s="28" t="inlineStr">
         <is>
-          <t>Modelo analítico, vistas, indicadores y guía reproducible completos; publicación productiva incluida en el Módulo 12.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -5213,14 +5213,14 @@
         <v>46311</v>
       </c>
       <c r="J119" s="30" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="K119" s="4" t="n">
         <v>15</v>
       </c>
       <c r="L119" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Parcial: las pruebas cubren los indicadores implementados; faltan los de humedad, temperatura y la comparación entre periodos.</t>
         </is>
       </c>
     </row>
@@ -5262,7 +5262,7 @@
       </c>
       <c r="L120" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -5300,7 +5300,7 @@
       </c>
       <c r="L121" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -5338,7 +5338,7 @@
       </c>
       <c r="L122" s="28" t="inlineStr">
         <is>
-          <t>Completado y validado en el cierre de software del 12/09/2026.</t>
+          <t>Adelantada: implementada antes del inicio planificado. El código está en el repositorio desde el 17/08/2026 y se validó en el cierre de software del 12/09/2026.</t>
         </is>
       </c>
     </row>
@@ -5800,12 +5800,12 @@
     <mergeCell ref="C109:C111"/>
     <mergeCell ref="C80:C84"/>
     <mergeCell ref="D113:D114"/>
-    <mergeCell ref="D35:D36"/>
     <mergeCell ref="D69:D70"/>
     <mergeCell ref="B46:B56"/>
     <mergeCell ref="C68:C71"/>
     <mergeCell ref="B123:B128"/>
     <mergeCell ref="A129:A131"/>
+    <mergeCell ref="D35:D36"/>
     <mergeCell ref="D116:D118"/>
     <mergeCell ref="C75:C79"/>
     <mergeCell ref="C18:C21"/>

</xml_diff>